<commit_message>
add EuroSys'27 HADIS publication
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10510"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huiguan/Documents/projects/website/guanh01.github.io/markdown_generator/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15BF59C-E369-D14C-9663-B6A6BF281763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="443">
   <si>
     <t>pub_date</t>
   </si>
@@ -175,6 +169,9 @@
     <t>2026-07-01</t>
   </si>
   <si>
+    <t>2027-04-01</t>
+  </si>
+  <si>
     <t>Hui Guan, Wen Tang, Hamid Krim, James Keiser, Andrew Rindos, and Radmila Sazdanovic</t>
   </si>
   <si>
@@ -347,6 +344,9 @@
   </si>
   <si>
     <t>Kunjal Panchal, Saayan Mitra, Sunav Choudhary, Victor Bursztyn, Somdeb Sarkhel, Hui Guan</t>
+  </si>
+  <si>
+    <t>Qizheng Yang, Tung-I Chen, Siyu Zhao, Ramesh K. Sitaraman, and Hui Guan</t>
   </si>
   <si>
     <t>A topological collapse for document summarization</t>
@@ -533,6 +533,9 @@
     <t>Mosaic: Runtime-Efficient Multi-Agent Embodied Planning</t>
   </si>
   <si>
+    <t>HADIS: Hybrid Adaptive Diffusion Model Serving for Efficient Text-to-Image Generation</t>
+  </si>
+  <si>
     <t>In 2016 IEEE 17th International Workshop on Signal Processing Advances in Wireless Communications (SPAWC), pp. 1-5. IEEE, 2016</t>
   </si>
   <si>
@@ -710,6 +713,9 @@
     <t>The 43rd International Conference on Machine Learning (ICML 2026), 2026</t>
   </si>
   <si>
+    <t>The 22nd European Conference on Computer Systems (EuroSys 2027)</t>
+  </si>
+  <si>
     <t>spawc</t>
   </si>
   <si>
@@ -899,6 +905,9 @@
     <t>icml26-mosaic-runtime</t>
   </si>
   <si>
+    <t>eurosys27-hadis-hybrid</t>
+  </si>
+  <si>
     <t>http://guanh01.github.io/files/2016spawc.pdf</t>
   </si>
   <si>
@@ -1082,6 +1091,9 @@
     <t>https://icml.cc/virtual/2026/poster/62291</t>
   </si>
   <si>
+    <t>https://arxiv.org/abs/2509.00642</t>
+  </si>
+  <si>
     <t>SPAWC'16</t>
   </si>
   <si>
@@ -1256,6 +1268,9 @@
     <t>ICML'26</t>
   </si>
   <si>
+    <t>EuroSys'27</t>
+  </si>
+  <si>
     <t>https://github.com/zhanglijun95/TreeMTL</t>
   </si>
   <si>
@@ -1283,6 +1298,12 @@
     <t>https://github.com/Astuary/Spry</t>
   </si>
   <si>
+    <t>https://github.com/Astuary/Gradient_Estimation_Methods</t>
+  </si>
+  <si>
+    <t>https://zenodo.org/records/22900370</t>
+  </si>
+  <si>
     <t>Poster~&gt;https://crossfl2022.github.io/posters/Poster9.pdf</t>
   </si>
   <si>
@@ -1323,16 +1344,13 @@
   </si>
   <si>
     <t>agentic-systems</t>
-  </si>
-  <si>
-    <t>https://github.com/Astuary/Gradient_Estimation_Methods</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1408,21 +1426,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1460,7 +1470,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1494,7 +1504,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1529,10 +1538,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1705,14 +1713,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="55" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K65"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1747,1770 +1752,1801 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="G2" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="K2" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E3" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="G3" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="K3" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="G4" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="K4" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E5" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G5" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="K5" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E6" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="G6" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="K6" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D7" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="E7" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="G7" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="K7" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D8" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E8" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="G8" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="K8" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D9" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E9" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="G9" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="K9" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D10" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E10" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="G10" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="K10" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E11" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="G11" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="K11" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D12" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E12" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="G12" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="K12" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D13" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E13" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="G13" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="K13" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C14" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D14" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E14" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="G14" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="K14" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C15" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D15" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E15" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="G15" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="K15" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D16" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E16" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="G16" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="K16" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
       <c r="A17" t="s">
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D17" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E17" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="G17" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="K17" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="A18" t="s">
         <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D18" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E18" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="G18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="K18" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
       <c r="A19" t="s">
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C19" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D19" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E19" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="G19" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="K19" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" t="s">
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C20" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D20" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E20" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="G20" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="K20" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
       <c r="A21" t="s">
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D21" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E21" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="G21" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="K21" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="A22" t="s">
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D22" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E22" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="G22" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="K22" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
       <c r="A23" t="s">
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D23" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="E23" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="G23" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="I23" t="s">
-        <v>420</v>
+        <v>429</v>
       </c>
       <c r="K23" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" t="s">
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D24" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E24" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="G24" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="I24" t="s">
-        <v>421</v>
+        <v>430</v>
       </c>
       <c r="K24" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
       <c r="A25" t="s">
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C25" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D25" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E25" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="G25" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="K25" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="A26" t="s">
         <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D26" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E26" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="G26" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="I26" t="s">
-        <v>422</v>
+        <v>431</v>
       </c>
       <c r="K26" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
       <c r="A27" t="s">
         <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C27" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D27" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E27" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="G27" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="K27" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28" t="s">
         <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C28" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D28" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="E28" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="G28" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="K28" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11">
       <c r="A29" t="s">
         <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D29" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E29" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="G29" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="K29" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="A30" t="s">
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D30" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E30" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="G30" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="K30" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
       <c r="A31" t="s">
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D31" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E31" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="G31" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="K31" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32" t="s">
         <v>33</v>
       </c>
       <c r="B32" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C32" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D32" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E32" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="G32" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="K32" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" t="s">
         <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D33" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="E33" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="G33" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="K33" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" t="s">
         <v>34</v>
       </c>
       <c r="B34" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D34" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E34" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="G34" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="K34" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" t="s">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C35" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D35" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E35" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="G35" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="K35" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" t="s">
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D36" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E36" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="G36" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="K36" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11">
       <c r="A37" t="s">
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C37" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D37" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E37" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="G37" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>423</v>
+        <v>432</v>
       </c>
       <c r="K37" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="A38" t="s">
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C38" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D38" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E38" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="G38" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>424</v>
+        <v>433</v>
       </c>
       <c r="K38" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
       <c r="A39" t="s">
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C39" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D39" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="E39" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="G39" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="K39" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" t="s">
         <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C40" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D40" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E40" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="G40" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="K40" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
       <c r="A41" t="s">
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D41" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="E41" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="G41" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="K41" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
       <c r="A42" t="s">
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C42" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D42" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E42" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="G42" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="K42" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
       <c r="A43" t="s">
         <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C43" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D43" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E43" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="G43" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="K43" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" t="s">
         <v>40</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D44" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E44" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="G44" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="K44" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11">
       <c r="A45" t="s">
         <v>40</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D45" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E45" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="G45" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="K45" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
       <c r="A46" t="s">
         <v>40</v>
       </c>
       <c r="B46" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C46" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D46" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E46" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="G46" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="K46" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11">
       <c r="A47" t="s">
         <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C47" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D47" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E47" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="G47" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="K47" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11">
       <c r="A48" t="s">
         <v>41</v>
       </c>
       <c r="B48" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C48" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D48" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="E48" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="G48" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="K48" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11">
       <c r="A49" t="s">
         <v>41</v>
       </c>
       <c r="B49" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C49" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D49" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E49" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="G49" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="K49" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11">
       <c r="A50" t="s">
         <v>41</v>
       </c>
       <c r="B50" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C50" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D50" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E50" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="G50" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="K50" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11">
       <c r="A51" t="s">
         <v>42</v>
       </c>
       <c r="B51" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C51" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D51" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="E51" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="G51" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="K51" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11">
       <c r="A52" t="s">
         <v>42</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C52" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D52" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="E52" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="G52" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="K52" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11">
       <c r="A53" t="s">
         <v>42</v>
       </c>
       <c r="B53" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C53" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D53" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E53" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="G53" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="K53" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11">
       <c r="A54" t="s">
         <v>43</v>
       </c>
       <c r="B54" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C54" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D54" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E54" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="G54" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="K54" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11">
       <c r="A55" t="s">
         <v>44</v>
       </c>
       <c r="B55" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C55" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D55" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E55" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="G55" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
       <c r="K55" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11">
       <c r="A56" t="s">
         <v>45</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C56" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D56" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E56" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="G56" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="K56" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11">
       <c r="A57" t="s">
         <v>46</v>
       </c>
       <c r="B57" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C57" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D57" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E57" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="G57" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="K57" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11">
       <c r="A58" t="s">
         <v>47</v>
       </c>
       <c r="B58" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C58" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D58" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="E58" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="G58" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="K58" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11">
       <c r="A59" t="s">
         <v>48</v>
       </c>
       <c r="B59" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C59" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D59" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E59" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="G59" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="K59" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11">
       <c r="A60" t="s">
         <v>49</v>
       </c>
       <c r="B60" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C60" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D60" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E60" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="G60" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="K60" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11">
       <c r="A61" t="s">
         <v>49</v>
       </c>
       <c r="B61" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C61" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D61" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E61" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="G61" t="s">
-        <v>409</v>
+        <v>415</v>
       </c>
       <c r="K61" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11">
       <c r="A62" t="s">
         <v>50</v>
       </c>
       <c r="B62" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C62" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D62" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E62" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="G62" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="K62" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11">
       <c r="A63" t="s">
         <v>50</v>
       </c>
       <c r="B63" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C63" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D63" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E63" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="G63" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>434</v>
+        <v>427</v>
       </c>
       <c r="K63" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11">
       <c r="A64" t="s">
         <v>50</v>
       </c>
       <c r="B64" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C64" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D64" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E64" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="G64" t="s">
-        <v>410</v>
+        <v>416</v>
       </c>
       <c r="K64" t="s">
-        <v>432</v>
+        <v>441</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11">
+      <c r="A65" t="s">
+        <v>51</v>
+      </c>
+      <c r="B65" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" t="s">
+        <v>172</v>
+      </c>
+      <c r="D65" t="s">
+        <v>232</v>
+      </c>
+      <c r="E65" t="s">
+        <v>296</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="G65" t="s">
+        <v>417</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="K65" t="s">
+        <v>440</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="F6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="F7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="F9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="F10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="F11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="F12" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="F13" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="F14" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="F15" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="F16" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="F17" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="F18" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="F19" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="F20" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="F21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="F22" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="F23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="F24" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="H24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="F25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="F26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="F27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="F28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="H28" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="F29" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="H29" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="F30" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="F31" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="F32" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="F33" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="F34" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="H34" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="F35" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="F36" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="H36" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="F37" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="H37" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="J37" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="F38" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="H38" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="J38" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="F39" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="F40" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="H40" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="J40" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="F41" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="F42" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="F43" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="J43" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="F44" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="F45" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="F46" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="H46" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="F47" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="H47" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="F48" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="F49" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="F50" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="F51" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="F52" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="F53" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="F54" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="F55" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="F56" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="F57" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="F59" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="F60" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="F61" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="F62" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="F63" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="F64" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="H63" r:id="rId76" xr:uid="{89D19EAB-1DF0-B44A-9A08-ED94402A2C41}"/>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="F3" r:id="rId2"/>
+    <hyperlink ref="F4" r:id="rId3"/>
+    <hyperlink ref="F6" r:id="rId4"/>
+    <hyperlink ref="F7" r:id="rId5"/>
+    <hyperlink ref="F8" r:id="rId6"/>
+    <hyperlink ref="F9" r:id="rId7"/>
+    <hyperlink ref="F10" r:id="rId8"/>
+    <hyperlink ref="F11" r:id="rId9"/>
+    <hyperlink ref="F12" r:id="rId10"/>
+    <hyperlink ref="F13" r:id="rId11"/>
+    <hyperlink ref="F14" r:id="rId12"/>
+    <hyperlink ref="F15" r:id="rId13"/>
+    <hyperlink ref="F16" r:id="rId14"/>
+    <hyperlink ref="F17" r:id="rId15"/>
+    <hyperlink ref="F18" r:id="rId16"/>
+    <hyperlink ref="F19" r:id="rId17"/>
+    <hyperlink ref="F20" r:id="rId18"/>
+    <hyperlink ref="F21" r:id="rId19"/>
+    <hyperlink ref="F22" r:id="rId20"/>
+    <hyperlink ref="F23" r:id="rId21"/>
+    <hyperlink ref="F24" r:id="rId22"/>
+    <hyperlink ref="H24" r:id="rId23"/>
+    <hyperlink ref="F25" r:id="rId24"/>
+    <hyperlink ref="F26" r:id="rId25"/>
+    <hyperlink ref="F27" r:id="rId26"/>
+    <hyperlink ref="F28" r:id="rId27"/>
+    <hyperlink ref="H28" r:id="rId28"/>
+    <hyperlink ref="F29" r:id="rId29"/>
+    <hyperlink ref="H29" r:id="rId30"/>
+    <hyperlink ref="F30" r:id="rId31"/>
+    <hyperlink ref="F31" r:id="rId32"/>
+    <hyperlink ref="F32" r:id="rId33"/>
+    <hyperlink ref="F33" r:id="rId34"/>
+    <hyperlink ref="F34" r:id="rId35"/>
+    <hyperlink ref="H34" r:id="rId36"/>
+    <hyperlink ref="F35" r:id="rId37"/>
+    <hyperlink ref="F36" r:id="rId38"/>
+    <hyperlink ref="H36" r:id="rId39"/>
+    <hyperlink ref="F37" r:id="rId40"/>
+    <hyperlink ref="H37" r:id="rId41"/>
+    <hyperlink ref="J37" r:id="rId42"/>
+    <hyperlink ref="F38" r:id="rId43"/>
+    <hyperlink ref="H38" r:id="rId44"/>
+    <hyperlink ref="J38" r:id="rId45"/>
+    <hyperlink ref="F39" r:id="rId46"/>
+    <hyperlink ref="F40" r:id="rId47"/>
+    <hyperlink ref="H40" r:id="rId48"/>
+    <hyperlink ref="J40" r:id="rId49"/>
+    <hyperlink ref="F41" r:id="rId50"/>
+    <hyperlink ref="F42" r:id="rId51"/>
+    <hyperlink ref="F43" r:id="rId52"/>
+    <hyperlink ref="J43" r:id="rId53"/>
+    <hyperlink ref="F44" r:id="rId54"/>
+    <hyperlink ref="F45" r:id="rId55"/>
+    <hyperlink ref="F46" r:id="rId56"/>
+    <hyperlink ref="H46" r:id="rId57"/>
+    <hyperlink ref="F47" r:id="rId58"/>
+    <hyperlink ref="H47" r:id="rId59"/>
+    <hyperlink ref="F48" r:id="rId60"/>
+    <hyperlink ref="F49" r:id="rId61"/>
+    <hyperlink ref="F50" r:id="rId62"/>
+    <hyperlink ref="F51" r:id="rId63"/>
+    <hyperlink ref="F52" r:id="rId64"/>
+    <hyperlink ref="F53" r:id="rId65"/>
+    <hyperlink ref="F54" r:id="rId66"/>
+    <hyperlink ref="F55" r:id="rId67"/>
+    <hyperlink ref="F56" r:id="rId68"/>
+    <hyperlink ref="F57" r:id="rId69"/>
+    <hyperlink ref="F59" r:id="rId70"/>
+    <hyperlink ref="F60" r:id="rId71"/>
+    <hyperlink ref="F61" r:id="rId72"/>
+    <hyperlink ref="F62" r:id="rId73"/>
+    <hyperlink ref="F63" r:id="rId74"/>
+    <hyperlink ref="H63" r:id="rId75"/>
+    <hyperlink ref="F64" r:id="rId76"/>
+    <hyperlink ref="F65" r:id="rId77"/>
+    <hyperlink ref="H65" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
sync publication metadata with CV
- HADIS (EuroSys'27): use the accepted title, "A Hybrid Architecture for
  Query-Aware Diffusion Model Serving", and add the PacificVis'26 paper link
- FLEET (MLSys'20): restore missing author Seung-Hwan Lim
- TNNLS'23: "Architectures" -> "Architecture" in title
- AdapMTL (ACM MM'24): Jiaxun Tang -> Steven Jiaxun Tang
- Proteus (ASPLOS'24): Brain D. Friedman -> Brian D. Friedman
- tags: Neurocomputing@25 -> Neurocomputing'25,
  InformationSystems'21 -> Information Systems'21
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="444">
   <si>
     <t>pub_date</t>
   </si>
@@ -202,7 +202,7 @@
     <t>Hui Guan, Andrey Malevich, Jiyan Yang,  Jongsoo Park, and Hector Yuen</t>
   </si>
   <si>
-    <t>Hui Guan, Laxmikant Kishor Mokadam, Xipeng Shen, Robert Patton</t>
+    <t>Hui Guan, Laxmikant Kishor Mokadam, Xipeng Shen, Seung-Hwan Lim, Robert Patton</t>
   </si>
   <si>
     <t>Zifan Nan, Hui Guan, Xipeng Shen</t>
@@ -268,7 +268,7 @@
     <t>Qizheng Yang, Tianyi Yang, Mingcan Xiang, Lijun Zhang, Haoliang Wang, Marco Serafini, Hui Guan</t>
   </si>
   <si>
-    <t>Sohaib Ahmad, Hui Guan, Brain D. Friedman, Thomas Williams, Ramesh K. Sitaraman, Thomas Woo</t>
+    <t>Sohaib Ahmad, Hui Guan, Brian D. Friedman, Thomas Williams, Ramesh K. Sitaraman, Thomas Woo</t>
   </si>
   <si>
     <t>Xiao Liu, Lijun Zhang, Hui Guan</t>
@@ -283,7 +283,7 @@
     <t>Siddhant Garg, Lijun Zhang, Hui Guan</t>
   </si>
   <si>
-    <t>Mingcan Xiang, Jiaxun Tang, Qizheng Yang, Hui Guan, Tongping Liu</t>
+    <t>Mingcan Xiang, Steven Jiaxun Tang, Qizheng Yang, Hui Guan, Tongping Liu</t>
   </si>
   <si>
     <t>Jin Zhou, Hanmei Yang, Steven Jiaxun Tang, Mingcan Xiang, Hui Guan, Tongping Liu</t>
@@ -427,7 +427,7 @@
     <t>AutoMTL: A Programming Framework for Automating Efficient Multi-Task Learning</t>
   </si>
   <si>
-    <t>A Tree-Structured Multi-Task Model Architectures Recommendation System</t>
+    <t>A Tree-Structured Multi-Task Model Architecture Recommendation System</t>
   </si>
   <si>
     <t>NUMAlloc: A Faster NUMA Memory Allocator</t>
@@ -533,7 +533,7 @@
     <t>Mosaic: Runtime-Efficient Multi-Agent Embodied Planning</t>
   </si>
   <si>
-    <t>HADIS: Hybrid Adaptive Diffusion Model Serving for Efficient Text-to-Image Generation</t>
+    <t>HADIS: A Hybrid Architecture for Query-Aware Diffusion Model Serving</t>
   </si>
   <si>
     <t>In 2016 IEEE 17th International Workshop on Signal Processing Advances in Wireless Communications (SPAWC), pp. 1-5. IEEE, 2016</t>
@@ -1073,6 +1073,9 @@
     <t>https://arxiv.org/abs/2512.17108</t>
   </si>
   <si>
+    <t>https://ieeexplore.ieee.org/document/11558675</t>
+  </si>
+  <si>
     <t>https://arxiv.org/pdf/2406.08334</t>
   </si>
   <si>
@@ -1136,7 +1139,7 @@
     <t>CC'21</t>
   </si>
   <si>
-    <t>InformationSystems'21</t>
+    <t>Information Systems'21</t>
   </si>
   <si>
     <t>ICS'21</t>
@@ -1232,7 +1235,7 @@
     <t>CHI EA'25</t>
   </si>
   <si>
-    <t>Neurocomputing@25</t>
+    <t>Neurocomputing'25</t>
   </si>
   <si>
     <t>ARITH'25</t>
@@ -1772,10 +1775,10 @@
         <v>297</v>
       </c>
       <c r="G2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="K2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1798,10 +1801,10 @@
         <v>298</v>
       </c>
       <c r="G3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="K3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1824,10 +1827,10 @@
         <v>299</v>
       </c>
       <c r="G4" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="K4" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1847,10 +1850,10 @@
         <v>236</v>
       </c>
       <c r="G5" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="K5" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1873,10 +1876,10 @@
         <v>300</v>
       </c>
       <c r="G6" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="K6" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1899,10 +1902,10 @@
         <v>301</v>
       </c>
       <c r="G7" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="K7" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1925,10 +1928,10 @@
         <v>302</v>
       </c>
       <c r="G8" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="K8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1951,10 +1954,10 @@
         <v>303</v>
       </c>
       <c r="G9" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="K9" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1977,10 +1980,10 @@
         <v>304</v>
       </c>
       <c r="G10" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K10" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2003,10 +2006,10 @@
         <v>305</v>
       </c>
       <c r="G11" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K11" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2029,10 +2032,10 @@
         <v>306</v>
       </c>
       <c r="G12" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K12" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2055,10 +2058,10 @@
         <v>307</v>
       </c>
       <c r="G13" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K13" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2081,10 +2084,10 @@
         <v>308</v>
       </c>
       <c r="G14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K14" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2107,10 +2110,10 @@
         <v>309</v>
       </c>
       <c r="G15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="K15" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2133,10 +2136,10 @@
         <v>310</v>
       </c>
       <c r="G16" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K16" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2159,10 +2162,10 @@
         <v>311</v>
       </c>
       <c r="G17" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="K17" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2185,10 +2188,10 @@
         <v>312</v>
       </c>
       <c r="G18" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K18" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2211,10 +2214,10 @@
         <v>313</v>
       </c>
       <c r="G19" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="K19" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2237,10 +2240,10 @@
         <v>314</v>
       </c>
       <c r="G20" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="K20" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2263,10 +2266,10 @@
         <v>315</v>
       </c>
       <c r="G21" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="K21" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2289,10 +2292,10 @@
         <v>316</v>
       </c>
       <c r="G22" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K22" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2315,13 +2318,13 @@
         <v>317</v>
       </c>
       <c r="G23" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="I23" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="K23" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2344,16 +2347,16 @@
         <v>318</v>
       </c>
       <c r="G24" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="I24" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K24" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2376,10 +2379,10 @@
         <v>319</v>
       </c>
       <c r="G25" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="K25" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2402,13 +2405,13 @@
         <v>320</v>
       </c>
       <c r="G26" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="I26" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="K26" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2431,10 +2434,10 @@
         <v>321</v>
       </c>
       <c r="G27" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="K27" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2457,13 +2460,13 @@
         <v>322</v>
       </c>
       <c r="G28" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="K28" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2486,13 +2489,13 @@
         <v>323</v>
       </c>
       <c r="G29" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="K29" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2515,10 +2518,10 @@
         <v>324</v>
       </c>
       <c r="G30" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="K30" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2541,10 +2544,10 @@
         <v>325</v>
       </c>
       <c r="G31" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="K31" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2567,10 +2570,10 @@
         <v>326</v>
       </c>
       <c r="G32" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K32" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2593,10 +2596,10 @@
         <v>327</v>
       </c>
       <c r="G33" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="K33" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2619,13 +2622,13 @@
         <v>328</v>
       </c>
       <c r="G34" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="K34" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2648,10 +2651,10 @@
         <v>329</v>
       </c>
       <c r="G35" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K35" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2674,13 +2677,13 @@
         <v>330</v>
       </c>
       <c r="G36" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="K36" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2703,16 +2706,16 @@
         <v>331</v>
       </c>
       <c r="G37" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K37" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2735,16 +2738,16 @@
         <v>332</v>
       </c>
       <c r="G38" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K38" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2767,10 +2770,10 @@
         <v>333</v>
       </c>
       <c r="G39" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K39" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2793,16 +2796,16 @@
         <v>334</v>
       </c>
       <c r="G40" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="K40" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2825,10 +2828,10 @@
         <v>335</v>
       </c>
       <c r="G41" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K41" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2851,10 +2854,10 @@
         <v>336</v>
       </c>
       <c r="G42" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="K42" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2877,13 +2880,13 @@
         <v>337</v>
       </c>
       <c r="G43" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="K43" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2906,10 +2909,10 @@
         <v>338</v>
       </c>
       <c r="G44" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K44" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2932,10 +2935,10 @@
         <v>339</v>
       </c>
       <c r="G45" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="K45" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -2958,13 +2961,13 @@
         <v>340</v>
       </c>
       <c r="G46" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K46" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -2987,13 +2990,13 @@
         <v>341</v>
       </c>
       <c r="G47" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K47" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3016,10 +3019,10 @@
         <v>342</v>
       </c>
       <c r="G48" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="K48" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3042,10 +3045,10 @@
         <v>343</v>
       </c>
       <c r="G49" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="K49" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3068,10 +3071,10 @@
         <v>344</v>
       </c>
       <c r="G50" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K50" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3094,10 +3097,10 @@
         <v>345</v>
       </c>
       <c r="G51" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K51" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3120,10 +3123,10 @@
         <v>346</v>
       </c>
       <c r="G52" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K52" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3146,10 +3149,10 @@
         <v>347</v>
       </c>
       <c r="G53" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="K53" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -3172,10 +3175,10 @@
         <v>348</v>
       </c>
       <c r="G54" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K54" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -3198,10 +3201,10 @@
         <v>349</v>
       </c>
       <c r="G55" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K55" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -3224,10 +3227,10 @@
         <v>350</v>
       </c>
       <c r="G56" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K56" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -3250,10 +3253,10 @@
         <v>351</v>
       </c>
       <c r="G57" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="K57" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -3272,11 +3275,14 @@
       <c r="E58" t="s">
         <v>289</v>
       </c>
+      <c r="F58" s="2" t="s">
+        <v>352</v>
+      </c>
       <c r="G58" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K58" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -3296,13 +3302,13 @@
         <v>290</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G59" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="K59" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -3322,13 +3328,13 @@
         <v>291</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G60" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="K60" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -3348,13 +3354,13 @@
         <v>292</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G61" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="K61" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3374,13 +3380,13 @@
         <v>293</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G62" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K62" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="63" spans="1:11">
@@ -3400,16 +3406,16 @@
         <v>294</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G63" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="K63" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -3429,13 +3435,13 @@
         <v>295</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G64" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="K64" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -3455,16 +3461,16 @@
         <v>296</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G65" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="K65" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -3538,15 +3544,16 @@
     <hyperlink ref="F55" r:id="rId67"/>
     <hyperlink ref="F56" r:id="rId68"/>
     <hyperlink ref="F57" r:id="rId69"/>
-    <hyperlink ref="F59" r:id="rId70"/>
-    <hyperlink ref="F60" r:id="rId71"/>
-    <hyperlink ref="F61" r:id="rId72"/>
-    <hyperlink ref="F62" r:id="rId73"/>
-    <hyperlink ref="F63" r:id="rId74"/>
-    <hyperlink ref="H63" r:id="rId75"/>
-    <hyperlink ref="F64" r:id="rId76"/>
-    <hyperlink ref="F65" r:id="rId77"/>
-    <hyperlink ref="H65" r:id="rId78"/>
+    <hyperlink ref="F58" r:id="rId70"/>
+    <hyperlink ref="F59" r:id="rId71"/>
+    <hyperlink ref="F60" r:id="rId72"/>
+    <hyperlink ref="F61" r:id="rId73"/>
+    <hyperlink ref="F62" r:id="rId74"/>
+    <hyperlink ref="F63" r:id="rId75"/>
+    <hyperlink ref="H63" r:id="rId76"/>
+    <hyperlink ref="F64" r:id="rId77"/>
+    <hyperlink ref="F65" r:id="rId78"/>
+    <hyperlink ref="H65" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>